<commit_message>
Update Base Class capabilities
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/01_Login/CompanyLogin/02_InfluencerLogin.xlsx
+++ b/src/test/resources/testdata/Modules/01_Login/CompanyLogin/02_InfluencerLogin.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\01_Login\CompanyLogin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E4B9845-AB3B-4DCD-A637-74907948302C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11E1DF13-F6AD-4750-A968-24BFB770F741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
@@ -74,9 +74,6 @@
     <t>1111</t>
   </si>
   <si>
-    <t>1234567891</t>
-  </si>
-  <si>
     <t>Navigate to Login page</t>
   </si>
   <si>
@@ -187,6 +184,9 @@
   </si>
   <si>
     <t>01_CompanyLogin</t>
+  </si>
+  <si>
+    <t>9527812704</t>
   </si>
 </sst>
 </file>
@@ -1173,21 +1173,21 @@
         <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
       <c r="H2" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>5</v>
@@ -1198,21 +1198,21 @@
         <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
       <c r="H3" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>5</v>
@@ -1223,23 +1223,23 @@
         <v>8</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>5</v>
@@ -1250,23 +1250,23 @@
         <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="9" t="s">
         <v>44</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>13</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>5</v>
@@ -1277,21 +1277,21 @@
         <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
       <c r="H6" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>5</v>
@@ -1302,23 +1302,23 @@
         <v>8</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>5</v>
@@ -1329,21 +1329,21 @@
         <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>5</v>
@@ -1354,23 +1354,23 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="E9" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1" t="s">
         <v>12</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>5</v>

</xml_diff>